<commit_message>
Update Excel model to final version
</commit_message>
<xml_diff>
--- a/model/excel/CPRT_short_model.xlsx
+++ b/model/excel/CPRT_short_model.xlsx
@@ -48,7 +48,7 @@
     <definedName name="MLNKe9251677bd324e0499c283d41b67cd36" hidden="1">Summary!$AH$49:$AP$59</definedName>
     <definedName name="MLNKfc765725f4964ce18842637b929224b1" hidden="1">'Financial Model'!$C$3:$M$42</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Assumptions'!$B$2:$H$10,'Assumptions'!$J$2:$R$16</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Model Notes'!$B$2:$L$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Model Notes'!$B$2:$L$17</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Summary'!$B$2:$U$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Summary Charts'!$B$2:$J$30,'Summary Charts'!$K$32:$V$49</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Historical Financials'!$B$2:$K$124</definedName>
@@ -4339,54 +4339,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>1</col>
-      <colOff>19051</colOff>
-      <row>4</row>
-      <rowOff>178733</rowOff>
-    </from>
-    <to>
-      <col>6</col>
-      <colOff>1</colOff>
-      <row>11</row>
-      <rowOff>29020</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Picture 4"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="624169" y="895909"/>
-          <a:ext cx="3006538" cy="1105346"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>1</col>
@@ -4939,7 +4891,6 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -13055,9 +13006,9 @@
         <f>('Financial Model'!T9*(1-T204)-'Financial Model'!T13-'Financial Model'!T24-SUM('Financial Model'!T30:T31)-T206)/T21</f>
         <v/>
       </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>Facility cost is the residual that delivers the operating-margin driver (row 204): cost per car rises faster than revenue per car.</t>
+      <c r="V22" s="360" t="inlineStr">
+        <is>
+          <t>This row carries the margin drop: 44.2% to 46.9% of service revenue in FY27E. It is the residual that delivers row 204. Base case: facility cost +$122M (+7.0%) on 3% fewer cars; per car, cost +10.3% vs revenue +4.0% (Q4 FY26 US: +14.2%).</t>
         </is>
       </c>
     </row>
@@ -13301,6 +13252,11 @@
         <f>$J$27</f>
         <v/>
       </c>
+      <c r="V27" s="360" t="inlineStr">
+        <is>
+          <t>Held at FY26 (88.5% of vehicle sales): not a source of the margin drop.</t>
+        </is>
+      </c>
     </row>
     <row r="28" outlineLevel="1" ht="14.25" customFormat="1" customHeight="1" s="8" thickBot="1">
       <c r="A28" s="7" t="n"/>
@@ -13564,6 +13520,11 @@
         <f>$J$33</f>
         <v/>
       </c>
+      <c r="V33" s="360" t="inlineStr">
+        <is>
+          <t>Held at FY26 (8.6% of revenue): not a source of the FY27E drop. G&amp;A took 263bp of margin FY23A-FY26A (6.0% to 8.6%).</t>
+        </is>
+      </c>
     </row>
     <row r="34" outlineLevel="1" ht="14.25" customFormat="1" customHeight="1" s="8">
       <c r="A34" s="7" t="n"/>
@@ -14292,9 +14253,9 @@
         <f>($J$46/'Financial Model'!$I$59)*'Financial Model'!S59/T48</f>
         <v/>
       </c>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>D&amp;A at FY26 rate on opening net PP&amp;E (yards do not shrink with units).</t>
+      <c r="V49" s="360" t="inlineStr">
+        <is>
+          <t>D&amp;A at FY26 rate on opening net PP&amp;E (yards do not shrink with units). Rises from 5.1% to 5.8% of revenue by FY30E, absorbed inside the flat operating margin.</t>
         </is>
       </c>
     </row>
@@ -20829,9 +20790,9 @@
         <f>S204+T205</f>
         <v/>
       </c>
-      <c r="V204" t="inlineStr">
-        <is>
-          <t>FY27E 33.0% memo Exhibit 2 (Q4 FY26 exit 32.0%); held flat - no margin recovery in printed case.</t>
+      <c r="V204" s="360" t="inlineStr">
+        <is>
+          <t>FY27E 33.0% memo Exhibit 2, then held flat. Not a new leg down: FY26A 35.4% blends 36.5% for the first nine months with a 32.0% Q4 exit, so 33.0% is 100bp above the exit rate. +100bp = ~$0.04 EPS, ~$0.61 on the target.</t>
         </is>
       </c>
     </row>
@@ -20867,6 +20828,11 @@
       </c>
       <c r="T205" s="742" t="n">
         <v>0</v>
+      </c>
+      <c r="V205" s="360" t="inlineStr">
+        <is>
+          <t>No recovery: units grow only +0.5% a year from FY30E, so no volume re-absorbs yard cost. Management says it will cut cost per car but gives no guidance: no credit given. Enter a step here to flex. See Model Notes 3-4.</t>
+        </is>
       </c>
     </row>
     <row r="206">
@@ -38026,7 +37992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G205"/>
+  <dimension ref="B2:G206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="2" max="2"/>
@@ -44266,6 +44232,38 @@
       <c r="G205" s="916" t="inlineStr">
         <is>
           <t>https://fred.stlouisfed.org/series/BAMLC0A0CMEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="B206" s="916" t="inlineStr">
+        <is>
+          <t>Model Notes 3-4; Drivers V22, V204, V205 margin facts</t>
+        </is>
+      </c>
+      <c r="C206" s="916" t="inlineStr">
+        <is>
+          <t>Q4 op income 368.9 (-10.6%); US facility cost +7.7%, +14.2% per unit; US units -5.7%; long-haul delivery 17</t>
+        </is>
+      </c>
+      <c r="D206" s="916" t="inlineStr">
+        <is>
+          <t>Q4 FY26</t>
+        </is>
+      </c>
+      <c r="E206" s="916" t="inlineStr">
+        <is>
+          <t>Q4 FY26 earnings call transcript</t>
+        </is>
+      </c>
+      <c r="F206" s="916" t="inlineStr">
+        <is>
+          <t>CFO prepared remarks and Q&amp;A (cost per car; no cost or margin guidance)</t>
+        </is>
+      </c>
+      <c r="G206" s="916" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/earnings/call-transcripts/2026/09/11/copart-cprt-q4-2026-earnings-call-transcript/</t>
         </is>
       </c>
     </row>
@@ -44580,12 +44578,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C3:K14"/>
+  <dimension ref="C3:K16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="12.75" zeroHeight="1"/>
   <cols>
     <col width="1.59765625" customWidth="1" min="1" max="1"/>
     <col width="1.73046875" customWidth="1" min="2" max="2"/>
-    <col width="8.73046875" customWidth="1" min="3" max="11"/>
+    <col width="8.73046875" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -44645,7 +44643,7 @@
       </c>
       <c r="D7" s="620" t="inlineStr">
         <is>
-          <t>Variant view: Street has FY27 EPS $1.75 (+11% per memo) and treats 17.6x vs a 34x ten-year median as a cyclical dip. Model FY27E EPS $1.44, 18% below; Street is a reference cell only (Support!D10). Unlike prior 30%+ drawdowns, trailing EPS is falling.</t>
+          <t>Margin path (what drops). Operating margin (Drivers row 204): 38.4% FY23A, 37.1%, 36.5%, 35.4% FY26A, 33.0% FY27E. FY23A-FY26A, -300bp of revenue: G&amp;A +263bp, facility operations +206bp, D&amp;A +98bp, less cost of vehicle sales -267bp. FY26A-FY27E, -242bp: facility operations +227bp, D&amp;A +15bp; G&amp;A and cost of vehicle sales held at FY26 rates. Cause: a growing cost base serves fewer cars. Q4 FY26 US facility cost rose 7.7% on 5.7% fewer US cars (+14.2% per car); management cites long-haul delivery ($17M of the increase), Title Express, wholesale yards and new capacity. Base FY27E: facility cost +$122M (+7.0%) on 3% fewer cars; cost per car +10.3% vs revenue per car +4.0%.</t>
         </is>
       </c>
     </row>
@@ -44656,7 +44654,7 @@
       </c>
       <c r="D8" s="620" t="inlineStr">
         <is>
-          <t>Falsifiers: cover if collision frequency is positive for two quarters; the lost-customer lap is already in the -3% unit assumption; catastrophe volume is excluded from the trend; stop reference $32.60 (above the 50-day and the 23.6% retracement). Short interest 4.6% of float is context, not an input.</t>
+          <t>Margin path (why 33.0%, and why it holds). FY27E is not a new leg down: FY26A's 35.4% blends 36.5% for the first nine months with a 32.0% Q4 exit ($368.9M / $1,152.4M), so 33.0% sits 100bp above the exit rate. Held to FY36E (Drivers row 205 = 0): units grow only +0.5% a year from FY30E, so no volume re-absorbs yard cost. Management says it will cut cost per car but gives no guidance; no credit given. +100bp of FY27E margin = ~$47M EBIT, ~$0.04 EPS, ~$0.61 on the target; bull case 36.5% = FY25A level. Net margin falls more (31.8% to 28.5%) as interest income drops from $182M to $110M after the ACV payment.</t>
         </is>
       </c>
     </row>
@@ -44667,7 +44665,7 @@
       </c>
       <c r="D9" s="620" t="inlineStr">
         <is>
-          <t>Catalysts: Q1 FY27 on Nov 19, 2026 (Street $0.40 vs $0.41); RB Global Q3 in early Nov; ACV close by year-end 2026; monthly CCC / insurer claim prints.</t>
+          <t>Variant view: Street has FY27 EPS $1.75 (+11% per memo) and treats 17.6x vs a 34x ten-year median as a cyclical dip. Model FY27E EPS $1.44, 18% below; Street is a reference cell only (Support!D10). Unlike prior 30%+ drawdowns, trailing EPS is falling.</t>
         </is>
       </c>
     </row>
@@ -44678,7 +44676,7 @@
       </c>
       <c r="D10" s="620" t="inlineStr">
         <is>
-          <t>Column map (no columns inserted): G = FY2023A (year ended July 31, 2023), H = FY2024A, I = FY2025A, J = FY2026A / LTM (July 31, 2026), K-T = FY2027E-FY2036E. Pitch window FY27E-FY31E; FY32E-FY36E fade (units +0.5%, revenue per unit to +1.5%, margin flat). DCF columns G-P = FY27E-FY36E. Units: $ millions except per share; shares in millions.</t>
+          <t>Falsifiers: cover if collision frequency is positive for two quarters; the lost-customer lap is already in the -3% unit assumption; catastrophe volume is excluded from the trend; stop reference $32.60 (above the 50-day and the 23.6% retracement). Short interest 4.6% of float is context, not an input.</t>
         </is>
       </c>
     </row>
@@ -44689,7 +44687,7 @@
       </c>
       <c r="D11" s="620" t="inlineStr">
         <is>
-          <t>Definitions. Cash = cash, equivalents, restricted cash + held-to-maturity securities ($4,489.8M FY26). Debt = revolver + term loan = 0; finance leases are not split out on the balance sheet (immaterial) and sit in lease liabilities. Capex and buybacks are negative (template sign). Net income = attributable to Copart: NCI loss runs through Other (Income)/Expense, so template EBT = reported pre-tax income + NCI loss ($3.9M FY26). Facility operations and G&amp;A include their SBC; D&amp;A is the cash-flow-statement total, so template gross profit is before D&amp;A (reported FY26 gross profit $2,083.9M = template $2,294.6M - $201.7M facility D&amp;A - $9.1M).</t>
+          <t>Catalysts: Q1 FY27 on Nov 19, 2026 (Street $0.40 vs $0.41); RB Global Q3 in early Nov; ACV close by year-end 2026; monthly CCC / insurer claim prints.</t>
         </is>
       </c>
     </row>
@@ -44700,7 +44698,7 @@
       </c>
       <c r="D12" s="620" t="inlineStr">
         <is>
-          <t>Filing vs memo flags. ACV: 8-K says ~$1.9B equity value; memo ~$1.8B; model uses $1.9B. Revenue $4,666M (memo $4.67B), operating income $1,652.6M, EPS $1.55, buybacks $1,632.5M, interest income net $181.9M: all tie. EV/EBITDA on CFS D&amp;A is 11.0x vs memo 11.1x. Street growth is +12.8% on $1.55, memo says +11%. Memo Exhibit 2 base target is $21.54 vs headline $21.50. Bull EPS computes to $1.67 vs memo $1.70 (see Support row 35). Unit levels are an index on the memo 4.0M base; Copart discloses growth rates only.</t>
+          <t>Column map (no columns inserted): G = FY2023A (year ended July 31, 2023), H = FY2024A, I = FY2025A, J = FY2026A / LTM (July 31, 2026), K-T = FY2027E-FY2036E. Pitch window FY27E-FY31E; FY32E-FY36E fade (units +0.5%, revenue per unit to +1.5%, margin flat). DCF columns G-P = FY27E-FY36E. Units: $ millions except per share; shares in millions.</t>
         </is>
       </c>
     </row>
@@ -44711,7 +44709,7 @@
       </c>
       <c r="D13" s="620" t="inlineStr">
         <is>
-          <t>Template formula changes (logged, none to force a result): first forecast column rolls from J (FY26A) instead of I; EPS row on Multiples &amp; Ratios was market cap / shares, now net income / shares; Summary FCF rows for interest, other and taxes now subtract; Financial Model H127:I127, Drivers G148:J148 (pointed at retained earnings) and L150:T150 reference fixes; LBO management rollover made non-circular; historical reconciling line (row 131) closes the derived cash-flow statement in FY23-FY26 only; DCF cost of debt and capital structure are inputs per brief; LBO cash is after ACV and row 83 excludes acquisitions; Comps stats wrapped in IFERROR.</t>
+          <t>Definitions. Cash = cash, equivalents, restricted cash + held-to-maturity securities ($4,489.8M FY26). Debt = revolver + term loan = 0; finance leases are not split out on the balance sheet (immaterial) and sit in lease liabilities. Capex and buybacks are negative (template sign). Net income = attributable to Copart: NCI loss runs through Other (Income)/Expense, so template EBT = reported pre-tax income + NCI loss ($3.9M FY26). Facility operations and G&amp;A include their SBC; D&amp;A is the cash-flow-statement total, so template gross profit is before D&amp;A (reported FY26 gross profit $2,083.9M = template $2,294.6M - $201.7M facility D&amp;A - $9.1M).</t>
         </is>
       </c>
     </row>
@@ -44722,17 +44720,41 @@
       </c>
       <c r="D14" s="620" t="inlineStr">
         <is>
+          <t>Filing vs memo flags. ACV: 8-K says ~$1.9B equity value; memo ~$1.8B; model uses $1.9B. Revenue $4,666M (memo $4.67B), operating income $1,652.6M, EPS $1.55, buybacks $1,632.5M, interest income net $181.9M: all tie. EV/EBITDA on CFS D&amp;A is 11.0x vs memo 11.1x. Street growth is +12.8% on $1.55, memo says +11%. Memo Exhibit 2 base target is $21.54 vs headline $21.50. Bull EPS computes to $1.67 vs memo $1.70 (see Support row 35). Unit levels are an index on the memo 4.0M base; Copart discloses growth rates only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="66" customHeight="1">
+      <c r="C15" s="188">
+        <f>+C14+1</f>
+        <v/>
+      </c>
+      <c r="D15" s="620" t="inlineStr">
+        <is>
+          <t>Template formula changes (logged, none to force a result): first forecast column rolls from J (FY26A) instead of I; EPS row on Multiples &amp; Ratios was market cap / shares, now net income / shares; Summary FCF rows for interest, other and taxes now subtract; Financial Model H127:I127, Drivers G148:J148 (pointed at retained earnings) and L150:T150 reference fixes; LBO management rollover made non-circular; historical reconciling line (row 131) closes the derived cash-flow statement in FY23-FY26 only; DCF cost of debt and capital structure are inputs per brief; LBO cash is after ACV and row 83 excludes acquisitions; Comps stats wrapped in IFERROR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="66" customHeight="1">
+      <c r="C16" s="188">
+        <f>+C15+1</f>
+        <v/>
+      </c>
+      <c r="D16" s="620" t="inlineStr">
+        <is>
           <t>Open items left blank and flagged, not invented: OPENLANE multiples and RBA / LKQ full comps lines as of Sep 30, 2026 (only memo forward P/Es loaded); ACV EV and profit measure (not in the 8-K); gross PP&amp;E / accumulated depreciation split; FY23 unit KPIs; IAA unit forecast (KPI 3 forecast = n/a); 2-year weekly beta not re-estimated (1.0 per brief); 10-K cover share count. DCF vs target and LBO IRR: see Support rows 88-116.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="10.05" customHeight="1"/>
+    <row r="17" ht="10.05" customHeight="1"/>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="12">
     <mergeCell ref="D9:K9"/>
     <mergeCell ref="D7:K7"/>
     <mergeCell ref="D8:K8"/>
     <mergeCell ref="D6:K6"/>
+    <mergeCell ref="D15:K15"/>
+    <mergeCell ref="D16:K16"/>
     <mergeCell ref="D11:K11"/>
     <mergeCell ref="D10:K10"/>
     <mergeCell ref="D14:K14"/>

</xml_diff>